<commit_message>
Feat: Added lot to XL data GUI
</commit_message>
<xml_diff>
--- a/DFR Transfer Log.xlsx
+++ b/DFR Transfer Log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming Local\WIPTrack Helper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF68B25C-2DBD-4926-BE00-A8D29AFD1429}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10C03E07-BDAB-4780-AD8B-DF99961D4EDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-16455" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Form1" sheetId="1" r:id="rId1"/>
@@ -95,8 +95,9 @@
 OperationNum - Note4</t>
   </si>
   <si>
-    <t>1404000 - Note 1
-1403200 - Note2</t>
+    <t>1404000 - Adding automation test 2 OP Number 1404000 Step 2
+1403200 - Adding automation test 2 OP Number 1403200 Step 3
+100 - Adding automation test 2 OP Number 100 Step 7</t>
   </si>
 </sst>
 </file>
@@ -731,7 +732,7 @@
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
     </row>
-    <row r="3" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:16" ht="72" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>

</xml_diff>